<commit_message>
docs: modify the complete dataset dictionary
</commit_message>
<xml_diff>
--- a/data/processed/dictionary_complete_dataset.xlsx
+++ b/data/processed/dictionary_complete_dataset.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Alvaro\amp_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C553D50-6FD1-4578-800E-2EE605BC3BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF48919F-D8B0-44E6-9B27-A5DA341D4678}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4338B850-6C41-46B1-9107-B422817CF49E}"/>
   </bookViews>
@@ -97,15 +97,9 @@
     <t>TrEMBL_ID</t>
   </si>
   <si>
-    <t>TrEMBL identifier from UniProt (unreviewed sequences)</t>
-  </si>
-  <si>
     <t>TrEMBL_name</t>
   </si>
   <si>
-    <t>Descriptive name from TrEMBL (UniProt)</t>
-  </si>
-  <si>
     <t>From_UniProt_in_ABPs</t>
   </si>
   <si>
@@ -590,6 +584,12 @@
   </si>
   <si>
     <t>Inferred Grand Average of Hidropathy (GRAVY) according to Kyte and Doolittle (1982)</t>
+  </si>
+  <si>
+    <t>TrEMBL identifier from UniProt (unreviewed sequences). Exists only if # ABPs for evaluation &gt; # reviewed non-AMPs for evaluation</t>
+  </si>
+  <si>
+    <t>Descriptive name from TrEMBL (UniProt). Exists only if # ABPs for evaluation &gt; # reviewed non-AMPs for evaluation</t>
   </si>
 </sst>
 </file>
@@ -1436,7 +1436,7 @@
   <cols>
     <col min="1" max="1" width="25.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="77.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="108.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -1568,887 +1568,887 @@
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>25</v>
+        <v>188</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
         <v>4</v>
       </c>
       <c r="C13" t="s">
-        <v>27</v>
+        <v>189</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" t="s">
         <v>28</v>
-      </c>
-      <c r="B14" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B15" t="s">
         <v>4</v>
       </c>
       <c r="C15" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" t="s">
         <v>33</v>
-      </c>
-      <c r="B16" t="s">
-        <v>34</v>
-      </c>
-      <c r="C16" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B17" t="s">
         <v>4</v>
       </c>
       <c r="C17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B18" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B19" t="s">
         <v>4</v>
       </c>
       <c r="C19" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B20" t="s">
         <v>4</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" t="s">
         <v>42</v>
-      </c>
-      <c r="B21" t="s">
-        <v>43</v>
-      </c>
-      <c r="C21" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B22" t="s">
         <v>4</v>
       </c>
       <c r="C22" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C23" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B24" t="s">
         <v>4</v>
       </c>
       <c r="C24" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B26" t="s">
         <v>4</v>
       </c>
       <c r="C26" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B27" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B28" t="s">
         <v>4</v>
       </c>
       <c r="C28" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B29" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C29" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B30" t="s">
         <v>4</v>
       </c>
       <c r="C30" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B31" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C31" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B32" t="s">
         <v>4</v>
       </c>
       <c r="C32" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B33" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C33" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B34" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C34" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B35" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B36" t="s">
         <v>4</v>
       </c>
       <c r="C36" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B37" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C37" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B38" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C38" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B39" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C39" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B40" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C40" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B41" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C41" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B42" t="s">
         <v>4</v>
       </c>
       <c r="C42" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B43" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C43" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B44" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C44" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B45" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C45" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B46" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C46" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B47" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C47" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
+        <v>91</v>
+      </c>
+      <c r="B48" t="s">
+        <v>92</v>
+      </c>
+      <c r="C48" t="s">
         <v>93</v>
-      </c>
-      <c r="B48" t="s">
-        <v>94</v>
-      </c>
-      <c r="C48" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B49" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C49" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B50" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C50" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B51" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C51" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B52" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C52" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B53" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C53" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B54" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C54" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B55" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C55" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B56" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C56" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B57" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C57" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B58" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C58" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B59" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C59" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B60" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C60" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B61" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C61" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B62" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C62" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B63" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C63" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B64" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C64" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B65" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C65" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B66" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C66" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B67" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C67" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B68" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C68" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B69" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C69" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B70" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C70" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B71" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C71" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B72" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C72" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B73" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C73" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B74" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C74" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B75" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C75" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B76" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C76" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B77" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C77" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B78" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C78" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B79" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C79" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B80" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C80" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B81" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C81" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B82" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C82" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B83" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C83" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B84" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C84" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B85" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C85" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B86" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C86" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B87" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C87" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B88" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C88" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B89" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C89" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B90" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C90" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B91" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C91" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B92" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C92" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>